<commit_message>
Atualiza a página com o caso real e a revisão humana
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/tabela-extracao-revisao.xlsx
+++ b/downloads/tabela-extracao-revisao.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,8 +44,14 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000E3D5F"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +61,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="000E3D5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A1C62E"/>
       </patternFill>
     </fill>
   </fills>
@@ -84,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -92,6 +103,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -842,7 +856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -852,6 +866,7 @@
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -895,6 +910,11 @@
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Conferido por</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Caso de fronteira decidido por (especialista)</t>
         </is>
       </c>
     </row>
@@ -906,6 +926,7 @@
       <c r="E3" s="3" t="n"/>
       <c r="F3" s="3" t="n"/>
       <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -915,6 +936,7 @@
       <c r="E4" s="3" t="n"/>
       <c r="F4" s="3" t="n"/>
       <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
@@ -924,6 +946,7 @@
       <c r="E5" s="3" t="n"/>
       <c r="F5" s="3" t="n"/>
       <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -933,6 +956,7 @@
       <c r="E6" s="3" t="n"/>
       <c r="F6" s="3" t="n"/>
       <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -942,6 +966,7 @@
       <c r="E7" s="3" t="n"/>
       <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -951,6 +976,7 @@
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="3" t="n"/>
       <c r="G8" s="3" t="n"/>
+      <c r="H8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -960,6 +986,7 @@
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="3" t="n"/>
       <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -969,6 +996,7 @@
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
+      <c r="H10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -978,6 +1006,7 @@
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -987,6 +1016,7 @@
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="n"/>
+      <c r="H12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -996,6 +1026,7 @@
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n"/>
       <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -1005,6 +1036,7 @@
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
       <c r="G14" s="3" t="n"/>
+      <c r="H14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -1014,6 +1046,7 @@
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -1023,6 +1056,7 @@
       <c r="E16" s="3" t="n"/>
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
+      <c r="H16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -1032,6 +1066,7 @@
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -1041,6 +1076,7 @@
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
       <c r="G18" s="3" t="n"/>
+      <c r="H18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -1050,6 +1086,7 @@
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -1059,6 +1096,7 @@
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="3" t="n"/>
+      <c r="H20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -1068,6 +1106,7 @@
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n"/>
+      <c r="H21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -1077,6 +1116,7 @@
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -1086,6 +1126,7 @@
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
       <c r="G23" s="3" t="n"/>
+      <c r="H23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -1095,6 +1136,7 @@
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
       <c r="G24" s="3" t="n"/>
+      <c r="H24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -1104,6 +1146,7 @@
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -1113,6 +1156,7 @@
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="n"/>
       <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -1122,6 +1166,7 @@
       <c r="E27" s="3" t="n"/>
       <c r="F27" s="3" t="n"/>
       <c r="G27" s="3" t="n"/>
+      <c r="H27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -1131,6 +1176,7 @@
       <c r="E28" s="3" t="n"/>
       <c r="F28" s="3" t="n"/>
       <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
@@ -1140,6 +1186,7 @@
       <c r="E29" s="3" t="n"/>
       <c r="F29" s="3" t="n"/>
       <c r="G29" s="3" t="n"/>
+      <c r="H29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -1149,6 +1196,7 @@
       <c r="E30" s="3" t="n"/>
       <c r="F30" s="3" t="n"/>
       <c r="G30" s="3" t="n"/>
+      <c r="H30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
@@ -1158,6 +1206,7 @@
       <c r="E31" s="3" t="n"/>
       <c r="F31" s="3" t="n"/>
       <c r="G31" s="3" t="n"/>
+      <c r="H31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -1167,6 +1216,7 @@
       <c r="E32" s="3" t="n"/>
       <c r="F32" s="3" t="n"/>
       <c r="G32" s="3" t="n"/>
+      <c r="H32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
@@ -1176,6 +1226,7 @@
       <c r="E33" s="3" t="n"/>
       <c r="F33" s="3" t="n"/>
       <c r="G33" s="3" t="n"/>
+      <c r="H33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -1185,6 +1236,7 @@
       <c r="E34" s="3" t="n"/>
       <c r="F34" s="3" t="n"/>
       <c r="G34" s="3" t="n"/>
+      <c r="H34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
@@ -1194,6 +1246,7 @@
       <c r="E35" s="3" t="n"/>
       <c r="F35" s="3" t="n"/>
       <c r="G35" s="3" t="n"/>
+      <c r="H35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -1203,6 +1256,7 @@
       <c r="E36" s="3" t="n"/>
       <c r="F36" s="3" t="n"/>
       <c r="G36" s="3" t="n"/>
+      <c r="H36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
@@ -1212,6 +1266,7 @@
       <c r="E37" s="3" t="n"/>
       <c r="F37" s="3" t="n"/>
       <c r="G37" s="3" t="n"/>
+      <c r="H37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -1221,6 +1276,7 @@
       <c r="E38" s="3" t="n"/>
       <c r="F38" s="3" t="n"/>
       <c r="G38" s="3" t="n"/>
+      <c r="H38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
@@ -1230,6 +1286,7 @@
       <c r="E39" s="3" t="n"/>
       <c r="F39" s="3" t="n"/>
       <c r="G39" s="3" t="n"/>
+      <c r="H39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -1239,6 +1296,7 @@
       <c r="E40" s="3" t="n"/>
       <c r="F40" s="3" t="n"/>
       <c r="G40" s="3" t="n"/>
+      <c r="H40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
@@ -1248,6 +1306,7 @@
       <c r="E41" s="3" t="n"/>
       <c r="F41" s="3" t="n"/>
       <c r="G41" s="3" t="n"/>
+      <c r="H41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -1257,6 +1316,7 @@
       <c r="E42" s="3" t="n"/>
       <c r="F42" s="3" t="n"/>
       <c r="G42" s="3" t="n"/>
+      <c r="H42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n"/>
@@ -1266,6 +1326,7 @@
       <c r="E43" s="3" t="n"/>
       <c r="F43" s="3" t="n"/>
       <c r="G43" s="3" t="n"/>
+      <c r="H43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
@@ -1275,6 +1336,7 @@
       <c r="E44" s="3" t="n"/>
       <c r="F44" s="3" t="n"/>
       <c r="G44" s="3" t="n"/>
+      <c r="H44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n"/>
@@ -1284,6 +1346,7 @@
       <c r="E45" s="3" t="n"/>
       <c r="F45" s="3" t="n"/>
       <c r="G45" s="3" t="n"/>
+      <c r="H45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
@@ -1293,6 +1356,7 @@
       <c r="E46" s="3" t="n"/>
       <c r="F46" s="3" t="n"/>
       <c r="G46" s="3" t="n"/>
+      <c r="H46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n"/>
@@ -1302,6 +1366,7 @@
       <c r="E47" s="3" t="n"/>
       <c r="F47" s="3" t="n"/>
       <c r="G47" s="3" t="n"/>
+      <c r="H47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -1311,6 +1376,7 @@
       <c r="E48" s="3" t="n"/>
       <c r="F48" s="3" t="n"/>
       <c r="G48" s="3" t="n"/>
+      <c r="H48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n"/>
@@ -1320,6 +1386,7 @@
       <c r="E49" s="3" t="n"/>
       <c r="F49" s="3" t="n"/>
       <c r="G49" s="3" t="n"/>
+      <c r="H49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
@@ -1329,6 +1396,7 @@
       <c r="E50" s="3" t="n"/>
       <c r="F50" s="3" t="n"/>
       <c r="G50" s="3" t="n"/>
+      <c r="H50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n"/>
@@ -1338,6 +1406,7 @@
       <c r="E51" s="3" t="n"/>
       <c r="F51" s="3" t="n"/>
       <c r="G51" s="3" t="n"/>
+      <c r="H51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
@@ -1347,6 +1416,7 @@
       <c r="E52" s="3" t="n"/>
       <c r="F52" s="3" t="n"/>
       <c r="G52" s="3" t="n"/>
+      <c r="H52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n"/>
@@ -1356,6 +1426,7 @@
       <c r="E53" s="3" t="n"/>
       <c r="F53" s="3" t="n"/>
       <c r="G53" s="3" t="n"/>
+      <c r="H53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
@@ -1365,6 +1436,7 @@
       <c r="E54" s="3" t="n"/>
       <c r="F54" s="3" t="n"/>
       <c r="G54" s="3" t="n"/>
+      <c r="H54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n"/>
@@ -1374,6 +1446,7 @@
       <c r="E55" s="3" t="n"/>
       <c r="F55" s="3" t="n"/>
       <c r="G55" s="3" t="n"/>
+      <c r="H55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
@@ -1383,6 +1456,7 @@
       <c r="E56" s="3" t="n"/>
       <c r="F56" s="3" t="n"/>
       <c r="G56" s="3" t="n"/>
+      <c r="H56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n"/>
@@ -1392,6 +1466,7 @@
       <c r="E57" s="3" t="n"/>
       <c r="F57" s="3" t="n"/>
       <c r="G57" s="3" t="n"/>
+      <c r="H57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
@@ -1401,6 +1476,7 @@
       <c r="E58" s="3" t="n"/>
       <c r="F58" s="3" t="n"/>
       <c r="G58" s="3" t="n"/>
+      <c r="H58" s="3" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n"/>
@@ -1410,6 +1486,7 @@
       <c r="E59" s="3" t="n"/>
       <c r="F59" s="3" t="n"/>
       <c r="G59" s="3" t="n"/>
+      <c r="H59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
@@ -1419,6 +1496,7 @@
       <c r="E60" s="3" t="n"/>
       <c r="F60" s="3" t="n"/>
       <c r="G60" s="3" t="n"/>
+      <c r="H60" s="3" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n"/>
@@ -1428,6 +1506,7 @@
       <c r="E61" s="3" t="n"/>
       <c r="F61" s="3" t="n"/>
       <c r="G61" s="3" t="n"/>
+      <c r="H61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
@@ -1437,6 +1516,7 @@
       <c r="E62" s="3" t="n"/>
       <c r="F62" s="3" t="n"/>
       <c r="G62" s="3" t="n"/>
+      <c r="H62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n"/>
@@ -1446,6 +1526,7 @@
       <c r="E63" s="3" t="n"/>
       <c r="F63" s="3" t="n"/>
       <c r="G63" s="3" t="n"/>
+      <c r="H63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
@@ -1455,6 +1536,7 @@
       <c r="E64" s="3" t="n"/>
       <c r="F64" s="3" t="n"/>
       <c r="G64" s="3" t="n"/>
+      <c r="H64" s="3" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n"/>
@@ -1464,6 +1546,7 @@
       <c r="E65" s="3" t="n"/>
       <c r="F65" s="3" t="n"/>
       <c r="G65" s="3" t="n"/>
+      <c r="H65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
@@ -1473,6 +1556,7 @@
       <c r="E66" s="3" t="n"/>
       <c r="F66" s="3" t="n"/>
       <c r="G66" s="3" t="n"/>
+      <c r="H66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n"/>
@@ -1482,6 +1566,7 @@
       <c r="E67" s="3" t="n"/>
       <c r="F67" s="3" t="n"/>
       <c r="G67" s="3" t="n"/>
+      <c r="H67" s="3" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n"/>
@@ -1491,6 +1576,7 @@
       <c r="E68" s="3" t="n"/>
       <c r="F68" s="3" t="n"/>
       <c r="G68" s="3" t="n"/>
+      <c r="H68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n"/>
@@ -1500,6 +1586,7 @@
       <c r="E69" s="3" t="n"/>
       <c r="F69" s="3" t="n"/>
       <c r="G69" s="3" t="n"/>
+      <c r="H69" s="3" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n"/>
@@ -1509,6 +1596,7 @@
       <c r="E70" s="3" t="n"/>
       <c r="F70" s="3" t="n"/>
       <c r="G70" s="3" t="n"/>
+      <c r="H70" s="3" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n"/>
@@ -1518,6 +1606,7 @@
       <c r="E71" s="3" t="n"/>
       <c r="F71" s="3" t="n"/>
       <c r="G71" s="3" t="n"/>
+      <c r="H71" s="3" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n"/>
@@ -1527,6 +1616,7 @@
       <c r="E72" s="3" t="n"/>
       <c r="F72" s="3" t="n"/>
       <c r="G72" s="3" t="n"/>
+      <c r="H72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n"/>
@@ -1536,6 +1626,7 @@
       <c r="E73" s="3" t="n"/>
       <c r="F73" s="3" t="n"/>
       <c r="G73" s="3" t="n"/>
+      <c r="H73" s="3" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n"/>
@@ -1545,6 +1636,7 @@
       <c r="E74" s="3" t="n"/>
       <c r="F74" s="3" t="n"/>
       <c r="G74" s="3" t="n"/>
+      <c r="H74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n"/>
@@ -1554,6 +1646,7 @@
       <c r="E75" s="3" t="n"/>
       <c r="F75" s="3" t="n"/>
       <c r="G75" s="3" t="n"/>
+      <c r="H75" s="3" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n"/>
@@ -1563,6 +1656,7 @@
       <c r="E76" s="3" t="n"/>
       <c r="F76" s="3" t="n"/>
       <c r="G76" s="3" t="n"/>
+      <c r="H76" s="3" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n"/>
@@ -1572,6 +1666,7 @@
       <c r="E77" s="3" t="n"/>
       <c r="F77" s="3" t="n"/>
       <c r="G77" s="3" t="n"/>
+      <c r="H77" s="3" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n"/>
@@ -1581,6 +1676,7 @@
       <c r="E78" s="3" t="n"/>
       <c r="F78" s="3" t="n"/>
       <c r="G78" s="3" t="n"/>
+      <c r="H78" s="3" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n"/>
@@ -1590,6 +1686,7 @@
       <c r="E79" s="3" t="n"/>
       <c r="F79" s="3" t="n"/>
       <c r="G79" s="3" t="n"/>
+      <c r="H79" s="3" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n"/>
@@ -1599,6 +1696,7 @@
       <c r="E80" s="3" t="n"/>
       <c r="F80" s="3" t="n"/>
       <c r="G80" s="3" t="n"/>
+      <c r="H80" s="3" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n"/>
@@ -1608,6 +1706,7 @@
       <c r="E81" s="3" t="n"/>
       <c r="F81" s="3" t="n"/>
       <c r="G81" s="3" t="n"/>
+      <c r="H81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n"/>
@@ -1617,10 +1716,11 @@
       <c r="E82" s="3" t="n"/>
       <c r="F82" s="3" t="n"/>
       <c r="G82" s="3" t="n"/>
+      <c r="H82" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="D3:D82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -1640,7 +1740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:O42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1656,12 +1756,14 @@
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="36" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Uma linha por estudo. Toda célula preenchida tem página. O que não estiver no estudo: não informado.</t>
+          <t>Uma linha por estudo. Toda célula preenchida tem página. Colunas verdes: preenchidas pelo especialista, não pela IA.</t>
         </is>
       </c>
     </row>
@@ -1729,6 +1831,16 @@
       <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Conferido por</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>Qualidade do desenho (avaliação do especialista)</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>Peso na síntese (especialista)</t>
         </is>
       </c>
     </row>
@@ -1746,6 +1858,8 @@
       <c r="K3" s="3" t="n"/>
       <c r="L3" s="3" t="n"/>
       <c r="M3" s="3" t="n"/>
+      <c r="N3" s="3" t="n"/>
+      <c r="O3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -1761,6 +1875,8 @@
       <c r="K4" s="3" t="n"/>
       <c r="L4" s="3" t="n"/>
       <c r="M4" s="3" t="n"/>
+      <c r="N4" s="3" t="n"/>
+      <c r="O4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
@@ -1776,6 +1892,8 @@
       <c r="K5" s="3" t="n"/>
       <c r="L5" s="3" t="n"/>
       <c r="M5" s="3" t="n"/>
+      <c r="N5" s="3" t="n"/>
+      <c r="O5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -1791,6 +1909,8 @@
       <c r="K6" s="3" t="n"/>
       <c r="L6" s="3" t="n"/>
       <c r="M6" s="3" t="n"/>
+      <c r="N6" s="3" t="n"/>
+      <c r="O6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -1806,6 +1926,8 @@
       <c r="K7" s="3" t="n"/>
       <c r="L7" s="3" t="n"/>
       <c r="M7" s="3" t="n"/>
+      <c r="N7" s="3" t="n"/>
+      <c r="O7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -1821,6 +1943,8 @@
       <c r="K8" s="3" t="n"/>
       <c r="L8" s="3" t="n"/>
       <c r="M8" s="3" t="n"/>
+      <c r="N8" s="3" t="n"/>
+      <c r="O8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -1836,6 +1960,8 @@
       <c r="K9" s="3" t="n"/>
       <c r="L9" s="3" t="n"/>
       <c r="M9" s="3" t="n"/>
+      <c r="N9" s="3" t="n"/>
+      <c r="O9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -1851,6 +1977,8 @@
       <c r="K10" s="3" t="n"/>
       <c r="L10" s="3" t="n"/>
       <c r="M10" s="3" t="n"/>
+      <c r="N10" s="3" t="n"/>
+      <c r="O10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -1866,6 +1994,8 @@
       <c r="K11" s="3" t="n"/>
       <c r="L11" s="3" t="n"/>
       <c r="M11" s="3" t="n"/>
+      <c r="N11" s="3" t="n"/>
+      <c r="O11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -1881,6 +2011,8 @@
       <c r="K12" s="3" t="n"/>
       <c r="L12" s="3" t="n"/>
       <c r="M12" s="3" t="n"/>
+      <c r="N12" s="3" t="n"/>
+      <c r="O12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -1896,6 +2028,8 @@
       <c r="K13" s="3" t="n"/>
       <c r="L13" s="3" t="n"/>
       <c r="M13" s="3" t="n"/>
+      <c r="N13" s="3" t="n"/>
+      <c r="O13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -1911,6 +2045,8 @@
       <c r="K14" s="3" t="n"/>
       <c r="L14" s="3" t="n"/>
       <c r="M14" s="3" t="n"/>
+      <c r="N14" s="3" t="n"/>
+      <c r="O14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -1926,6 +2062,8 @@
       <c r="K15" s="3" t="n"/>
       <c r="L15" s="3" t="n"/>
       <c r="M15" s="3" t="n"/>
+      <c r="N15" s="3" t="n"/>
+      <c r="O15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -1941,6 +2079,8 @@
       <c r="K16" s="3" t="n"/>
       <c r="L16" s="3" t="n"/>
       <c r="M16" s="3" t="n"/>
+      <c r="N16" s="3" t="n"/>
+      <c r="O16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -1956,6 +2096,8 @@
       <c r="K17" s="3" t="n"/>
       <c r="L17" s="3" t="n"/>
       <c r="M17" s="3" t="n"/>
+      <c r="N17" s="3" t="n"/>
+      <c r="O17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -1971,6 +2113,8 @@
       <c r="K18" s="3" t="n"/>
       <c r="L18" s="3" t="n"/>
       <c r="M18" s="3" t="n"/>
+      <c r="N18" s="3" t="n"/>
+      <c r="O18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -1986,6 +2130,8 @@
       <c r="K19" s="3" t="n"/>
       <c r="L19" s="3" t="n"/>
       <c r="M19" s="3" t="n"/>
+      <c r="N19" s="3" t="n"/>
+      <c r="O19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -2001,6 +2147,8 @@
       <c r="K20" s="3" t="n"/>
       <c r="L20" s="3" t="n"/>
       <c r="M20" s="3" t="n"/>
+      <c r="N20" s="3" t="n"/>
+      <c r="O20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -2016,6 +2164,8 @@
       <c r="K21" s="3" t="n"/>
       <c r="L21" s="3" t="n"/>
       <c r="M21" s="3" t="n"/>
+      <c r="N21" s="3" t="n"/>
+      <c r="O21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -2031,6 +2181,8 @@
       <c r="K22" s="3" t="n"/>
       <c r="L22" s="3" t="n"/>
       <c r="M22" s="3" t="n"/>
+      <c r="N22" s="3" t="n"/>
+      <c r="O22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -2046,6 +2198,8 @@
       <c r="K23" s="3" t="n"/>
       <c r="L23" s="3" t="n"/>
       <c r="M23" s="3" t="n"/>
+      <c r="N23" s="3" t="n"/>
+      <c r="O23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -2061,6 +2215,8 @@
       <c r="K24" s="3" t="n"/>
       <c r="L24" s="3" t="n"/>
       <c r="M24" s="3" t="n"/>
+      <c r="N24" s="3" t="n"/>
+      <c r="O24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -2076,6 +2232,8 @@
       <c r="K25" s="3" t="n"/>
       <c r="L25" s="3" t="n"/>
       <c r="M25" s="3" t="n"/>
+      <c r="N25" s="3" t="n"/>
+      <c r="O25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -2091,6 +2249,8 @@
       <c r="K26" s="3" t="n"/>
       <c r="L26" s="3" t="n"/>
       <c r="M26" s="3" t="n"/>
+      <c r="N26" s="3" t="n"/>
+      <c r="O26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -2106,6 +2266,8 @@
       <c r="K27" s="3" t="n"/>
       <c r="L27" s="3" t="n"/>
       <c r="M27" s="3" t="n"/>
+      <c r="N27" s="3" t="n"/>
+      <c r="O27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -2121,6 +2283,8 @@
       <c r="K28" s="3" t="n"/>
       <c r="L28" s="3" t="n"/>
       <c r="M28" s="3" t="n"/>
+      <c r="N28" s="3" t="n"/>
+      <c r="O28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
@@ -2136,6 +2300,8 @@
       <c r="K29" s="3" t="n"/>
       <c r="L29" s="3" t="n"/>
       <c r="M29" s="3" t="n"/>
+      <c r="N29" s="3" t="n"/>
+      <c r="O29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -2151,6 +2317,8 @@
       <c r="K30" s="3" t="n"/>
       <c r="L30" s="3" t="n"/>
       <c r="M30" s="3" t="n"/>
+      <c r="N30" s="3" t="n"/>
+      <c r="O30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
@@ -2166,6 +2334,8 @@
       <c r="K31" s="3" t="n"/>
       <c r="L31" s="3" t="n"/>
       <c r="M31" s="3" t="n"/>
+      <c r="N31" s="3" t="n"/>
+      <c r="O31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -2181,6 +2351,8 @@
       <c r="K32" s="3" t="n"/>
       <c r="L32" s="3" t="n"/>
       <c r="M32" s="3" t="n"/>
+      <c r="N32" s="3" t="n"/>
+      <c r="O32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
@@ -2196,6 +2368,8 @@
       <c r="K33" s="3" t="n"/>
       <c r="L33" s="3" t="n"/>
       <c r="M33" s="3" t="n"/>
+      <c r="N33" s="3" t="n"/>
+      <c r="O33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -2211,6 +2385,8 @@
       <c r="K34" s="3" t="n"/>
       <c r="L34" s="3" t="n"/>
       <c r="M34" s="3" t="n"/>
+      <c r="N34" s="3" t="n"/>
+      <c r="O34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
@@ -2226,6 +2402,8 @@
       <c r="K35" s="3" t="n"/>
       <c r="L35" s="3" t="n"/>
       <c r="M35" s="3" t="n"/>
+      <c r="N35" s="3" t="n"/>
+      <c r="O35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -2241,6 +2419,8 @@
       <c r="K36" s="3" t="n"/>
       <c r="L36" s="3" t="n"/>
       <c r="M36" s="3" t="n"/>
+      <c r="N36" s="3" t="n"/>
+      <c r="O36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
@@ -2256,6 +2436,8 @@
       <c r="K37" s="3" t="n"/>
       <c r="L37" s="3" t="n"/>
       <c r="M37" s="3" t="n"/>
+      <c r="N37" s="3" t="n"/>
+      <c r="O37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -2271,6 +2453,8 @@
       <c r="K38" s="3" t="n"/>
       <c r="L38" s="3" t="n"/>
       <c r="M38" s="3" t="n"/>
+      <c r="N38" s="3" t="n"/>
+      <c r="O38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
@@ -2286,6 +2470,8 @@
       <c r="K39" s="3" t="n"/>
       <c r="L39" s="3" t="n"/>
       <c r="M39" s="3" t="n"/>
+      <c r="N39" s="3" t="n"/>
+      <c r="O39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -2301,6 +2487,8 @@
       <c r="K40" s="3" t="n"/>
       <c r="L40" s="3" t="n"/>
       <c r="M40" s="3" t="n"/>
+      <c r="N40" s="3" t="n"/>
+      <c r="O40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
@@ -2316,6 +2504,8 @@
       <c r="K41" s="3" t="n"/>
       <c r="L41" s="3" t="n"/>
       <c r="M41" s="3" t="n"/>
+      <c r="N41" s="3" t="n"/>
+      <c r="O41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -2331,12 +2521,15 @@
       <c r="K42" s="3" t="n"/>
       <c r="L42" s="3" t="n"/>
       <c r="M42" s="3" t="n"/>
+      <c r="N42" s="3" t="n"/>
+      <c r="O42" s="3" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="B3:B42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"artigo publicado,working paper,relatório"</formula1>
     </dataValidation>
@@ -2349,6 +2542,9 @@
     <dataValidation sqref="I3:I42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"média,subgrupo,não informado"</formula1>
     </dataValidation>
+    <dataValidation sqref="O3:O42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"alto,moderado,baixo"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2360,7 +2556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F62"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -2369,6 +2565,7 @@
     <col width="55" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2407,6 +2604,11 @@
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Correção feita</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Aprovado pelo especialista</t>
         </is>
       </c>
     </row>
@@ -2417,6 +2619,7 @@
       <c r="D3" s="3" t="n"/>
       <c r="E3" s="3" t="n"/>
       <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -2425,6 +2628,7 @@
       <c r="D4" s="3" t="n"/>
       <c r="E4" s="3" t="n"/>
       <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
@@ -2433,6 +2637,7 @@
       <c r="D5" s="3" t="n"/>
       <c r="E5" s="3" t="n"/>
       <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -2441,6 +2646,7 @@
       <c r="D6" s="3" t="n"/>
       <c r="E6" s="3" t="n"/>
       <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -2449,6 +2655,7 @@
       <c r="D7" s="3" t="n"/>
       <c r="E7" s="3" t="n"/>
       <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -2457,6 +2664,7 @@
       <c r="D8" s="3" t="n"/>
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -2465,6 +2673,7 @@
       <c r="D9" s="3" t="n"/>
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="3" t="n"/>
+      <c r="G9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -2473,6 +2682,7 @@
       <c r="D10" s="3" t="n"/>
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
+      <c r="G10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -2481,6 +2691,7 @@
       <c r="D11" s="3" t="n"/>
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n"/>
+      <c r="G11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -2489,6 +2700,7 @@
       <c r="D12" s="3" t="n"/>
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="n"/>
+      <c r="G12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -2497,6 +2709,7 @@
       <c r="D13" s="3" t="n"/>
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n"/>
+      <c r="G13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -2505,6 +2718,7 @@
       <c r="D14" s="3" t="n"/>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -2513,6 +2727,7 @@
       <c r="D15" s="3" t="n"/>
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -2521,6 +2736,7 @@
       <c r="D16" s="3" t="n"/>
       <c r="E16" s="3" t="n"/>
       <c r="F16" s="3" t="n"/>
+      <c r="G16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -2529,6 +2745,7 @@
       <c r="D17" s="3" t="n"/>
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -2537,6 +2754,7 @@
       <c r="D18" s="3" t="n"/>
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
+      <c r="G18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -2545,6 +2763,7 @@
       <c r="D19" s="3" t="n"/>
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
+      <c r="G19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -2553,6 +2772,7 @@
       <c r="D20" s="3" t="n"/>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
+      <c r="G20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -2561,6 +2781,7 @@
       <c r="D21" s="3" t="n"/>
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
+      <c r="G21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -2569,6 +2790,7 @@
       <c r="D22" s="3" t="n"/>
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -2577,6 +2799,7 @@
       <c r="D23" s="3" t="n"/>
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
+      <c r="G23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -2585,6 +2808,7 @@
       <c r="D24" s="3" t="n"/>
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
+      <c r="G24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -2593,6 +2817,7 @@
       <c r="D25" s="3" t="n"/>
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -2601,6 +2826,7 @@
       <c r="D26" s="3" t="n"/>
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -2609,6 +2835,7 @@
       <c r="D27" s="3" t="n"/>
       <c r="E27" s="3" t="n"/>
       <c r="F27" s="3" t="n"/>
+      <c r="G27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -2617,6 +2844,7 @@
       <c r="D28" s="3" t="n"/>
       <c r="E28" s="3" t="n"/>
       <c r="F28" s="3" t="n"/>
+      <c r="G28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
@@ -2625,6 +2853,7 @@
       <c r="D29" s="3" t="n"/>
       <c r="E29" s="3" t="n"/>
       <c r="F29" s="3" t="n"/>
+      <c r="G29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -2633,6 +2862,7 @@
       <c r="D30" s="3" t="n"/>
       <c r="E30" s="3" t="n"/>
       <c r="F30" s="3" t="n"/>
+      <c r="G30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
@@ -2641,6 +2871,7 @@
       <c r="D31" s="3" t="n"/>
       <c r="E31" s="3" t="n"/>
       <c r="F31" s="3" t="n"/>
+      <c r="G31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -2649,6 +2880,7 @@
       <c r="D32" s="3" t="n"/>
       <c r="E32" s="3" t="n"/>
       <c r="F32" s="3" t="n"/>
+      <c r="G32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
@@ -2657,6 +2889,7 @@
       <c r="D33" s="3" t="n"/>
       <c r="E33" s="3" t="n"/>
       <c r="F33" s="3" t="n"/>
+      <c r="G33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -2665,6 +2898,7 @@
       <c r="D34" s="3" t="n"/>
       <c r="E34" s="3" t="n"/>
       <c r="F34" s="3" t="n"/>
+      <c r="G34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
@@ -2673,6 +2907,7 @@
       <c r="D35" s="3" t="n"/>
       <c r="E35" s="3" t="n"/>
       <c r="F35" s="3" t="n"/>
+      <c r="G35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -2681,6 +2916,7 @@
       <c r="D36" s="3" t="n"/>
       <c r="E36" s="3" t="n"/>
       <c r="F36" s="3" t="n"/>
+      <c r="G36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
@@ -2689,6 +2925,7 @@
       <c r="D37" s="3" t="n"/>
       <c r="E37" s="3" t="n"/>
       <c r="F37" s="3" t="n"/>
+      <c r="G37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -2697,6 +2934,7 @@
       <c r="D38" s="3" t="n"/>
       <c r="E38" s="3" t="n"/>
       <c r="F38" s="3" t="n"/>
+      <c r="G38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
@@ -2705,6 +2943,7 @@
       <c r="D39" s="3" t="n"/>
       <c r="E39" s="3" t="n"/>
       <c r="F39" s="3" t="n"/>
+      <c r="G39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -2713,6 +2952,7 @@
       <c r="D40" s="3" t="n"/>
       <c r="E40" s="3" t="n"/>
       <c r="F40" s="3" t="n"/>
+      <c r="G40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
@@ -2721,6 +2961,7 @@
       <c r="D41" s="3" t="n"/>
       <c r="E41" s="3" t="n"/>
       <c r="F41" s="3" t="n"/>
+      <c r="G41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -2729,6 +2970,7 @@
       <c r="D42" s="3" t="n"/>
       <c r="E42" s="3" t="n"/>
       <c r="F42" s="3" t="n"/>
+      <c r="G42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n"/>
@@ -2737,6 +2979,7 @@
       <c r="D43" s="3" t="n"/>
       <c r="E43" s="3" t="n"/>
       <c r="F43" s="3" t="n"/>
+      <c r="G43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
@@ -2745,6 +2988,7 @@
       <c r="D44" s="3" t="n"/>
       <c r="E44" s="3" t="n"/>
       <c r="F44" s="3" t="n"/>
+      <c r="G44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n"/>
@@ -2753,6 +2997,7 @@
       <c r="D45" s="3" t="n"/>
       <c r="E45" s="3" t="n"/>
       <c r="F45" s="3" t="n"/>
+      <c r="G45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
@@ -2761,6 +3006,7 @@
       <c r="D46" s="3" t="n"/>
       <c r="E46" s="3" t="n"/>
       <c r="F46" s="3" t="n"/>
+      <c r="G46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n"/>
@@ -2769,6 +3015,7 @@
       <c r="D47" s="3" t="n"/>
       <c r="E47" s="3" t="n"/>
       <c r="F47" s="3" t="n"/>
+      <c r="G47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -2777,6 +3024,7 @@
       <c r="D48" s="3" t="n"/>
       <c r="E48" s="3" t="n"/>
       <c r="F48" s="3" t="n"/>
+      <c r="G48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n"/>
@@ -2785,6 +3033,7 @@
       <c r="D49" s="3" t="n"/>
       <c r="E49" s="3" t="n"/>
       <c r="F49" s="3" t="n"/>
+      <c r="G49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
@@ -2793,6 +3042,7 @@
       <c r="D50" s="3" t="n"/>
       <c r="E50" s="3" t="n"/>
       <c r="F50" s="3" t="n"/>
+      <c r="G50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n"/>
@@ -2801,6 +3051,7 @@
       <c r="D51" s="3" t="n"/>
       <c r="E51" s="3" t="n"/>
       <c r="F51" s="3" t="n"/>
+      <c r="G51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
@@ -2809,6 +3060,7 @@
       <c r="D52" s="3" t="n"/>
       <c r="E52" s="3" t="n"/>
       <c r="F52" s="3" t="n"/>
+      <c r="G52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n"/>
@@ -2817,6 +3069,7 @@
       <c r="D53" s="3" t="n"/>
       <c r="E53" s="3" t="n"/>
       <c r="F53" s="3" t="n"/>
+      <c r="G53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
@@ -2825,6 +3078,7 @@
       <c r="D54" s="3" t="n"/>
       <c r="E54" s="3" t="n"/>
       <c r="F54" s="3" t="n"/>
+      <c r="G54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n"/>
@@ -2833,6 +3087,7 @@
       <c r="D55" s="3" t="n"/>
       <c r="E55" s="3" t="n"/>
       <c r="F55" s="3" t="n"/>
+      <c r="G55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
@@ -2841,6 +3096,7 @@
       <c r="D56" s="3" t="n"/>
       <c r="E56" s="3" t="n"/>
       <c r="F56" s="3" t="n"/>
+      <c r="G56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n"/>
@@ -2849,6 +3105,7 @@
       <c r="D57" s="3" t="n"/>
       <c r="E57" s="3" t="n"/>
       <c r="F57" s="3" t="n"/>
+      <c r="G57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
@@ -2857,6 +3114,7 @@
       <c r="D58" s="3" t="n"/>
       <c r="E58" s="3" t="n"/>
       <c r="F58" s="3" t="n"/>
+      <c r="G58" s="3" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n"/>
@@ -2865,6 +3123,7 @@
       <c r="D59" s="3" t="n"/>
       <c r="E59" s="3" t="n"/>
       <c r="F59" s="3" t="n"/>
+      <c r="G59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
@@ -2873,6 +3132,7 @@
       <c r="D60" s="3" t="n"/>
       <c r="E60" s="3" t="n"/>
       <c r="F60" s="3" t="n"/>
+      <c r="G60" s="3" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n"/>
@@ -2881,6 +3141,7 @@
       <c r="D61" s="3" t="n"/>
       <c r="E61" s="3" t="n"/>
       <c r="F61" s="3" t="n"/>
+      <c r="G61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
@@ -2889,10 +3150,11 @@
       <c r="D62" s="3" t="n"/>
       <c r="E62" s="3" t="n"/>
       <c r="F62" s="3" t="n"/>
+      <c r="G62" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="E3:E62" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Regra de status de leitura e marcador [não encontrado]
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/tabela-extracao-revisao.xlsx
+++ b/downloads/tabela-extracao-revisao.xlsx
@@ -2537,10 +2537,10 @@
       <formula1>"mede efeito (com comparação),revisão ou meta-análise,descritivo"</formula1>
     </dataValidation>
     <dataValidation sqref="G3:G42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"houve efeito,não houve,inconclusivo,não informado"</formula1>
+      <formula1>"houve efeito,não houve,inconclusivo,[não encontrado]"</formula1>
     </dataValidation>
     <dataValidation sqref="I3:I42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"média,subgrupo,não informado"</formula1>
+      <formula1>"média,subgrupo,[não encontrado]"</formula1>
     </dataValidation>
     <dataValidation sqref="O3:O42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"alto,moderado,baixo"</formula1>

</xml_diff>

<commit_message>
Coluna de status de leitura na planilha, tabela e skill
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/tabela-extracao-revisao.xlsx
+++ b/downloads/tabela-extracao-revisao.xlsx
@@ -1740,30 +1740,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="36" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="36" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="36" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Uma linha por estudo. Toda célula preenchida tem página. Colunas verdes: preenchidas pelo especialista, não pela IA.</t>
+          <t>Uma linha por estudo. Toda célula preenchida tem página. Colunas verdes: preenchidas pelo especialista, não pela IA. Status de leitura: só estudo lido na íntegra sustenta resultado; os demais vão para a lista de pendências, com o motivo.</t>
         </is>
       </c>
     </row>
@@ -1775,70 +1776,75 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>Status de leitura</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
           <t>Versão</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Pergunta</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Desenho</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Amostra e contexto</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Desfecho e quando foi medido</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Efeito encontrado</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Magnitude (como no estudo)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Média ou subgrupo</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Limitações declaradas</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>Exemplo prático</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Páginas</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Conferido por</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>Qualidade do desenho (avaliação do especialista)</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>Peso na síntese (especialista)</t>
         </is>
@@ -1860,6 +1866,7 @@
       <c r="M3" s="3" t="n"/>
       <c r="N3" s="3" t="n"/>
       <c r="O3" s="3" t="n"/>
+      <c r="P3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -1877,6 +1884,7 @@
       <c r="M4" s="3" t="n"/>
       <c r="N4" s="3" t="n"/>
       <c r="O4" s="3" t="n"/>
+      <c r="P4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
@@ -1894,6 +1902,7 @@
       <c r="M5" s="3" t="n"/>
       <c r="N5" s="3" t="n"/>
       <c r="O5" s="3" t="n"/>
+      <c r="P5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -1911,6 +1920,7 @@
       <c r="M6" s="3" t="n"/>
       <c r="N6" s="3" t="n"/>
       <c r="O6" s="3" t="n"/>
+      <c r="P6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -1928,6 +1938,7 @@
       <c r="M7" s="3" t="n"/>
       <c r="N7" s="3" t="n"/>
       <c r="O7" s="3" t="n"/>
+      <c r="P7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -1945,6 +1956,7 @@
       <c r="M8" s="3" t="n"/>
       <c r="N8" s="3" t="n"/>
       <c r="O8" s="3" t="n"/>
+      <c r="P8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -1962,6 +1974,7 @@
       <c r="M9" s="3" t="n"/>
       <c r="N9" s="3" t="n"/>
       <c r="O9" s="3" t="n"/>
+      <c r="P9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -1979,6 +1992,7 @@
       <c r="M10" s="3" t="n"/>
       <c r="N10" s="3" t="n"/>
       <c r="O10" s="3" t="n"/>
+      <c r="P10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -1996,6 +2010,7 @@
       <c r="M11" s="3" t="n"/>
       <c r="N11" s="3" t="n"/>
       <c r="O11" s="3" t="n"/>
+      <c r="P11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -2013,6 +2028,7 @@
       <c r="M12" s="3" t="n"/>
       <c r="N12" s="3" t="n"/>
       <c r="O12" s="3" t="n"/>
+      <c r="P12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -2030,6 +2046,7 @@
       <c r="M13" s="3" t="n"/>
       <c r="N13" s="3" t="n"/>
       <c r="O13" s="3" t="n"/>
+      <c r="P13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -2047,6 +2064,7 @@
       <c r="M14" s="3" t="n"/>
       <c r="N14" s="3" t="n"/>
       <c r="O14" s="3" t="n"/>
+      <c r="P14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -2064,6 +2082,7 @@
       <c r="M15" s="3" t="n"/>
       <c r="N15" s="3" t="n"/>
       <c r="O15" s="3" t="n"/>
+      <c r="P15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -2081,6 +2100,7 @@
       <c r="M16" s="3" t="n"/>
       <c r="N16" s="3" t="n"/>
       <c r="O16" s="3" t="n"/>
+      <c r="P16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -2098,6 +2118,7 @@
       <c r="M17" s="3" t="n"/>
       <c r="N17" s="3" t="n"/>
       <c r="O17" s="3" t="n"/>
+      <c r="P17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -2115,6 +2136,7 @@
       <c r="M18" s="3" t="n"/>
       <c r="N18" s="3" t="n"/>
       <c r="O18" s="3" t="n"/>
+      <c r="P18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -2132,6 +2154,7 @@
       <c r="M19" s="3" t="n"/>
       <c r="N19" s="3" t="n"/>
       <c r="O19" s="3" t="n"/>
+      <c r="P19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -2149,6 +2172,7 @@
       <c r="M20" s="3" t="n"/>
       <c r="N20" s="3" t="n"/>
       <c r="O20" s="3" t="n"/>
+      <c r="P20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -2166,6 +2190,7 @@
       <c r="M21" s="3" t="n"/>
       <c r="N21" s="3" t="n"/>
       <c r="O21" s="3" t="n"/>
+      <c r="P21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -2183,6 +2208,7 @@
       <c r="M22" s="3" t="n"/>
       <c r="N22" s="3" t="n"/>
       <c r="O22" s="3" t="n"/>
+      <c r="P22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -2200,6 +2226,7 @@
       <c r="M23" s="3" t="n"/>
       <c r="N23" s="3" t="n"/>
       <c r="O23" s="3" t="n"/>
+      <c r="P23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -2217,6 +2244,7 @@
       <c r="M24" s="3" t="n"/>
       <c r="N24" s="3" t="n"/>
       <c r="O24" s="3" t="n"/>
+      <c r="P24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -2234,6 +2262,7 @@
       <c r="M25" s="3" t="n"/>
       <c r="N25" s="3" t="n"/>
       <c r="O25" s="3" t="n"/>
+      <c r="P25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -2251,6 +2280,7 @@
       <c r="M26" s="3" t="n"/>
       <c r="N26" s="3" t="n"/>
       <c r="O26" s="3" t="n"/>
+      <c r="P26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -2268,6 +2298,7 @@
       <c r="M27" s="3" t="n"/>
       <c r="N27" s="3" t="n"/>
       <c r="O27" s="3" t="n"/>
+      <c r="P27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -2285,6 +2316,7 @@
       <c r="M28" s="3" t="n"/>
       <c r="N28" s="3" t="n"/>
       <c r="O28" s="3" t="n"/>
+      <c r="P28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
@@ -2302,6 +2334,7 @@
       <c r="M29" s="3" t="n"/>
       <c r="N29" s="3" t="n"/>
       <c r="O29" s="3" t="n"/>
+      <c r="P29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -2319,6 +2352,7 @@
       <c r="M30" s="3" t="n"/>
       <c r="N30" s="3" t="n"/>
       <c r="O30" s="3" t="n"/>
+      <c r="P30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
@@ -2336,6 +2370,7 @@
       <c r="M31" s="3" t="n"/>
       <c r="N31" s="3" t="n"/>
       <c r="O31" s="3" t="n"/>
+      <c r="P31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -2353,6 +2388,7 @@
       <c r="M32" s="3" t="n"/>
       <c r="N32" s="3" t="n"/>
       <c r="O32" s="3" t="n"/>
+      <c r="P32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
@@ -2370,6 +2406,7 @@
       <c r="M33" s="3" t="n"/>
       <c r="N33" s="3" t="n"/>
       <c r="O33" s="3" t="n"/>
+      <c r="P33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -2387,6 +2424,7 @@
       <c r="M34" s="3" t="n"/>
       <c r="N34" s="3" t="n"/>
       <c r="O34" s="3" t="n"/>
+      <c r="P34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
@@ -2404,6 +2442,7 @@
       <c r="M35" s="3" t="n"/>
       <c r="N35" s="3" t="n"/>
       <c r="O35" s="3" t="n"/>
+      <c r="P35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -2421,6 +2460,7 @@
       <c r="M36" s="3" t="n"/>
       <c r="N36" s="3" t="n"/>
       <c r="O36" s="3" t="n"/>
+      <c r="P36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
@@ -2438,6 +2478,7 @@
       <c r="M37" s="3" t="n"/>
       <c r="N37" s="3" t="n"/>
       <c r="O37" s="3" t="n"/>
+      <c r="P37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -2455,6 +2496,7 @@
       <c r="M38" s="3" t="n"/>
       <c r="N38" s="3" t="n"/>
       <c r="O38" s="3" t="n"/>
+      <c r="P38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
@@ -2472,6 +2514,7 @@
       <c r="M39" s="3" t="n"/>
       <c r="N39" s="3" t="n"/>
       <c r="O39" s="3" t="n"/>
+      <c r="P39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -2489,6 +2532,7 @@
       <c r="M40" s="3" t="n"/>
       <c r="N40" s="3" t="n"/>
       <c r="O40" s="3" t="n"/>
+      <c r="P40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
@@ -2506,6 +2550,7 @@
       <c r="M41" s="3" t="n"/>
       <c r="N41" s="3" t="n"/>
       <c r="O41" s="3" t="n"/>
+      <c r="P41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -2523,26 +2568,30 @@
       <c r="M42" s="3" t="n"/>
       <c r="N42" s="3" t="n"/>
       <c r="O42" s="3" t="n"/>
+      <c r="P42" s="3" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A1:P1"/>
     <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A1:N1"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation sqref="B3:B42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"lido na íntegra,só resumo conferido,não acessado"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C3:C42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"artigo publicado,working paper,relatório"</formula1>
     </dataValidation>
-    <dataValidation sqref="D3:D42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E3:E42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"mede efeito (com comparação),revisão ou meta-análise,descritivo"</formula1>
     </dataValidation>
-    <dataValidation sqref="G3:G42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H3:H42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"houve efeito,não houve,inconclusivo,[não encontrado]"</formula1>
     </dataValidation>
-    <dataValidation sqref="I3:I42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J3:J42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"média,subgrupo,[não encontrado]"</formula1>
     </dataValidation>
-    <dataValidation sqref="O3:O42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P3:P42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"alto,moderado,baixo"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>